<commit_message>
Date the project 2026, data as of November 2025
</commit_message>
<xml_diff>
--- a/Ferrari_Credit_Application_Model.xlsx
+++ b/Ferrari_Credit_Application_Model.xlsx
@@ -36,16 +36,16 @@
     <t xml:space="preserve">Business Plan and Credit Assessment, 2022A-2030F</t>
   </si>
   <si>
-    <t xml:space="preserve">EM032 Banking, IES FSV UK</t>
+    <t xml:space="preserve">2026</t>
   </si>
   <si>
     <t xml:space="preserve">Matúš Balko</t>
   </si>
   <si>
-    <t xml:space="preserve">November 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hypothetical case study: the Ferrari Residential Complex Miami project, its costs, financing and loan terms are made up for an academic exercise. Ferrari N.V. has not announced such a project. Historical 2022-2024 figures are Ferrari's reported data.</t>
+    <t xml:space="preserve">Data as of November 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hypothetical case study: the Ferrari Residential Complex Miami project, its costs, financing and loan terms are fictional. Ferrari N.V. has not announced such a project. Historical 2022-2024 figures are Ferrari's reported data.</t>
   </si>
   <si>
     <t xml:space="preserve">Table of Contents</t>
@@ -162,7 +162,7 @@
     <t xml:space="preserve">Project interest is expensed through the income statement. This is a simplification, as under IAS 23 it would be capitalised into inventory and released on handover.</t>
   </si>
   <si>
-    <t xml:space="preserve">Hypothetical case study: the Miami residential project and the loan are fictional and were made up for an academic exercise. Not affiliated with or endorsed by Ferrari N.V.</t>
+    <t xml:space="preserve">Hypothetical case study: the Miami residential project and the loan are fictional. Not affiliated with or endorsed by Ferrari N.V.</t>
   </si>
   <si>
     <t xml:space="preserve">Ferrari N.V.  |  Credit Application Model</t>

</xml_diff>